<commit_message>
Refresh unrestricted formal Q4 results
</commit_message>
<xml_diff>
--- a/05_results/q4/result.xlsx
+++ b/05_results/q4/result.xlsx
@@ -423,7 +423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L10"/>
+  <dimension ref="A1:L53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="13.8"/>
   <cols>
     <col width="15.77734375" customWidth="1" min="4" max="4"/>
@@ -474,19 +474,19 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>S05</t>
+          <t>P17</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>射击</t>
+          <t>拍照</t>
         </is>
       </c>
       <c r="D2" t="n">
-        <v>450.31</v>
+        <v>445.01</v>
       </c>
       <c r="E2" t="n">
-        <v>451.81</v>
+        <v>445.51</v>
       </c>
       <c r="H2" s="1" t="inlineStr">
         <is>
@@ -504,7 +504,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>P04</t>
+          <t>P18</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -513,10 +513,10 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>454.61</v>
+        <v>445.01</v>
       </c>
       <c r="E3" t="n">
-        <v>455.11</v>
+        <v>445.51</v>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
@@ -550,7 +550,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>P09</t>
+          <t>P05</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -559,10 +559,10 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>455.21</v>
+        <v>445.11</v>
       </c>
       <c r="E4" t="n">
-        <v>455.71</v>
+        <v>445.61</v>
       </c>
       <c r="H4" s="2" t="n">
         <v>1</v>
@@ -590,7 +590,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>P12</t>
+          <t>P13</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -599,10 +599,10 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>456.01</v>
+        <v>450.81</v>
       </c>
       <c r="E5" t="n">
-        <v>456.51</v>
+        <v>451.31</v>
       </c>
       <c r="H5" s="3" t="n"/>
       <c r="I5" s="3" t="n"/>
@@ -616,19 +616,19 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>S04</t>
+          <t>P08</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>射击</t>
+          <t>拍照</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>464.21</v>
+        <v>451.11</v>
       </c>
       <c r="E6" t="n">
-        <v>465.71</v>
+        <v>451.61</v>
       </c>
     </row>
     <row r="7">
@@ -637,7 +637,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>P16</t>
+          <t>P14</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -646,10 +646,10 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>466.61</v>
+        <v>451.28</v>
       </c>
       <c r="E7" t="n">
-        <v>467.11</v>
+        <v>451.78</v>
       </c>
     </row>
     <row r="8">
@@ -658,19 +658,19 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>P03</t>
+          <t>S05</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>拍照</t>
+          <t>射击</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>493.21</v>
+        <v>450.29</v>
       </c>
       <c r="E8" t="n">
-        <v>493.71</v>
+        <v>451.79</v>
       </c>
     </row>
     <row r="9">
@@ -679,7 +679,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>S11</t>
+          <t>S07</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -688,10 +688,10 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>509.31</v>
+        <v>451.03</v>
       </c>
       <c r="E9" t="n">
-        <v>510.81</v>
+        <v>452.53</v>
       </c>
     </row>
     <row r="10">
@@ -700,19 +700,922 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
+          <t>P15</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>拍照</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>453.89</v>
+      </c>
+      <c r="E10" t="n">
+        <v>454.39</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>P04</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>拍照</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>454.6</v>
+      </c>
+      <c r="E11" t="n">
+        <v>455.1</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>P09</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>拍照</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>454.76</v>
+      </c>
+      <c r="E12" t="n">
+        <v>455.26</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>P12</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>拍照</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>455.22</v>
+      </c>
+      <c r="E13" t="n">
+        <v>455.72</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>S09</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>射击</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>459.73</v>
+      </c>
+      <c r="E14" t="n">
+        <v>461.23</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>P03</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>拍照</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>463.92</v>
+      </c>
+      <c r="E15" t="n">
+        <v>464.42</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>P11</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>拍照</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>463.94</v>
+      </c>
+      <c r="E16" t="n">
+        <v>464.44</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>P07</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>拍照</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>463.97</v>
+      </c>
+      <c r="E17" t="n">
+        <v>464.47</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>S08</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>射击</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>463.18</v>
+      </c>
+      <c r="E18" t="n">
+        <v>464.68</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>S04</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>射击</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>464.26</v>
+      </c>
+      <c r="E19" t="n">
+        <v>465.76</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>P16</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>拍照</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>466.7</v>
+      </c>
+      <c r="E20" t="n">
+        <v>467.2</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>P06</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>拍照</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>467.6</v>
+      </c>
+      <c r="E21" t="n">
+        <v>468.1</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>P04</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>拍照</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>477.36</v>
+      </c>
+      <c r="E22" t="n">
+        <v>477.86</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>P10</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>拍照</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>477.36</v>
+      </c>
+      <c r="E23" t="n">
+        <v>477.86</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>S06</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>射击</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>476.93</v>
+      </c>
+      <c r="E24" t="n">
+        <v>478.43</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>P14</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>拍照</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
+        <v>480.95</v>
+      </c>
+      <c r="E25" t="n">
+        <v>481.45</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>P01</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>拍照</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
+        <v>481.27</v>
+      </c>
+      <c r="E26" t="n">
+        <v>481.77</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="n">
+        <v>26</v>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>P02</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>拍照</t>
+        </is>
+      </c>
+      <c r="D27" t="n">
+        <v>481.27</v>
+      </c>
+      <c r="E27" t="n">
+        <v>481.77</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="n">
+        <v>27</v>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>P05</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>拍照</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>481.27</v>
+      </c>
+      <c r="E28" t="n">
+        <v>481.77</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="n">
+        <v>28</v>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>P06</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>拍照</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
+        <v>481.27</v>
+      </c>
+      <c r="E29" t="n">
+        <v>481.77</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="n">
+        <v>29</v>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>P12</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>拍照</t>
+        </is>
+      </c>
+      <c r="D30" t="n">
+        <v>481.27</v>
+      </c>
+      <c r="E30" t="n">
+        <v>481.77</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="n">
+        <v>30</v>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>P13</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>拍照</t>
+        </is>
+      </c>
+      <c r="D31" t="n">
+        <v>481.27</v>
+      </c>
+      <c r="E31" t="n">
+        <v>481.77</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="n">
+        <v>31</v>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>S01</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>射击</t>
+        </is>
+      </c>
+      <c r="D32" t="n">
+        <v>480.53</v>
+      </c>
+      <c r="E32" t="n">
+        <v>482.03</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="n">
+        <v>32</v>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>S03</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>射击</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>480.68</v>
+      </c>
+      <c r="E33" t="n">
+        <v>482.18</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="n">
+        <v>33</v>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>P02</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>拍照</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
+        <v>492.95</v>
+      </c>
+      <c r="E34" t="n">
+        <v>493.45</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="n">
+        <v>34</v>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>P10</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>拍照</t>
+        </is>
+      </c>
+      <c r="D35" t="n">
+        <v>492.99</v>
+      </c>
+      <c r="E35" t="n">
+        <v>493.49</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="n">
+        <v>35</v>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>P11</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>拍照</t>
+        </is>
+      </c>
+      <c r="D36" t="n">
+        <v>493.09</v>
+      </c>
+      <c r="E36" t="n">
+        <v>493.59</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="n">
+        <v>36</v>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>P03</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>拍照</t>
+        </is>
+      </c>
+      <c r="D37" t="n">
+        <v>493.13</v>
+      </c>
+      <c r="E37" t="n">
+        <v>493.63</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="n">
+        <v>37</v>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>S02</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>射击</t>
+        </is>
+      </c>
+      <c r="D38" t="n">
+        <v>492.78</v>
+      </c>
+      <c r="E38" t="n">
+        <v>494.28</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="n">
+        <v>38</v>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>P04</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>拍照</t>
+        </is>
+      </c>
+      <c r="D39" t="n">
+        <v>494.15</v>
+      </c>
+      <c r="E39" t="n">
+        <v>494.65</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="n">
+        <v>39</v>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>P01</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>拍照</t>
+        </is>
+      </c>
+      <c r="D40" t="n">
+        <v>508.39</v>
+      </c>
+      <c r="E40" t="n">
+        <v>508.89</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="n">
+        <v>40</v>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>P02</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>拍照</t>
+        </is>
+      </c>
+      <c r="D41" t="n">
+        <v>508.81</v>
+      </c>
+      <c r="E41" t="n">
+        <v>509.31</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="n">
+        <v>41</v>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>S11</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>射击</t>
+        </is>
+      </c>
+      <c r="D42" t="n">
+        <v>509.36</v>
+      </c>
+      <c r="E42" t="n">
+        <v>510.86</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="n">
+        <v>42</v>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
           <t>S10</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
+      <c r="C43" t="inlineStr">
         <is>
           <t>射击</t>
         </is>
       </c>
-      <c r="D10" t="n">
-        <v>525.51</v>
-      </c>
-      <c r="E10" t="n">
-        <v>527.01</v>
+      <c r="D43" t="n">
+        <v>525.53</v>
+      </c>
+      <c r="E43" t="n">
+        <v>527.03</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="n">
+        <v>43</v>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>P02</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>拍照</t>
+        </is>
+      </c>
+      <c r="D44" t="n">
+        <v>749.96</v>
+      </c>
+      <c r="E44" t="n">
+        <v>750.46</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="n">
+        <v>44</v>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>P07</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>拍照</t>
+        </is>
+      </c>
+      <c r="D45" t="n">
+        <v>750.33</v>
+      </c>
+      <c r="E45" t="n">
+        <v>750.83</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="n">
+        <v>45</v>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>P04</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>拍照</t>
+        </is>
+      </c>
+      <c r="D46" t="n">
+        <v>750.34</v>
+      </c>
+      <c r="E46" t="n">
+        <v>750.84</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="n">
+        <v>46</v>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>P05</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>拍照</t>
+        </is>
+      </c>
+      <c r="D47" t="n">
+        <v>750.34</v>
+      </c>
+      <c r="E47" t="n">
+        <v>750.84</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="n">
+        <v>47</v>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>P08</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>拍照</t>
+        </is>
+      </c>
+      <c r="D48" t="n">
+        <v>750.34</v>
+      </c>
+      <c r="E48" t="n">
+        <v>750.84</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="n">
+        <v>48</v>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>S14</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>射击</t>
+        </is>
+      </c>
+      <c r="D49" t="n">
+        <v>749.64</v>
+      </c>
+      <c r="E49" t="n">
+        <v>751.14</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="n">
+        <v>49</v>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>S16</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>射击</t>
+        </is>
+      </c>
+      <c r="D50" t="n">
+        <v>749.75</v>
+      </c>
+      <c r="E50" t="n">
+        <v>751.25</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="n">
+        <v>50</v>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>S15</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>射击</t>
+        </is>
+      </c>
+      <c r="D51" t="n">
+        <v>749.85</v>
+      </c>
+      <c r="E51" t="n">
+        <v>751.35</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="n">
+        <v>51</v>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>S13</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>射击</t>
+        </is>
+      </c>
+      <c r="D52" t="n">
+        <v>761.99</v>
+      </c>
+      <c r="E52" t="n">
+        <v>763.49</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="n">
+        <v>52</v>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>S12</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>射击</t>
+        </is>
+      </c>
+      <c r="D53" t="n">
+        <v>762.5700000000001</v>
+      </c>
+      <c r="E53" t="n">
+        <v>764.0700000000001</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: reproduce all results and finalize paper
</commit_message>
<xml_diff>
--- a/05_results/q4/result.xlsx
+++ b/05_results/q4/result.xlsx
@@ -1,12 +1,12 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="162913" fullCalcOnLoad="1"/>
@@ -423,7 +423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L10"/>
+  <dimension ref="A1:L41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="13.8"/>
   <cols>
     <col width="15.77734375" customWidth="1" min="4" max="4"/>
@@ -474,19 +474,19 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>S05</t>
+          <t>P17</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>射击</t>
+          <t>拍照</t>
         </is>
       </c>
       <c r="D2" t="n">
-        <v>450.31</v>
+        <v>445.01</v>
       </c>
       <c r="E2" t="n">
-        <v>451.81</v>
+        <v>445.51</v>
       </c>
       <c r="H2" s="1" t="inlineStr">
         <is>
@@ -504,19 +504,19 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>P04</t>
+          <t>S06</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>拍照</t>
+          <t>射击</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>454.61</v>
+        <v>446.01</v>
       </c>
       <c r="E3" t="n">
-        <v>455.11</v>
+        <v>447.51</v>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
@@ -550,19 +550,19 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>P09</t>
+          <t>S05</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>拍照</t>
+          <t>射击</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>455.21</v>
+        <v>448.01</v>
       </c>
       <c r="E4" t="n">
-        <v>455.71</v>
+        <v>449.51</v>
       </c>
       <c r="H4" s="2" t="n">
         <v>1</v>
@@ -590,7 +590,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>P12</t>
+          <t>P18</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -599,10 +599,10 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>456.01</v>
+        <v>450.21</v>
       </c>
       <c r="E5" t="n">
-        <v>456.51</v>
+        <v>450.71</v>
       </c>
       <c r="H5" s="3" t="n"/>
       <c r="I5" s="3" t="n"/>
@@ -616,19 +616,19 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>S04</t>
+          <t>P08</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>射击</t>
+          <t>拍照</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>464.21</v>
+        <v>450.91</v>
       </c>
       <c r="E6" t="n">
-        <v>465.71</v>
+        <v>451.41</v>
       </c>
     </row>
     <row r="7">
@@ -637,7 +637,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>P16</t>
+          <t>P14</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -646,10 +646,10 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>466.61</v>
+        <v>451.51</v>
       </c>
       <c r="E7" t="n">
-        <v>467.11</v>
+        <v>452.01</v>
       </c>
     </row>
     <row r="8">
@@ -658,7 +658,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>P03</t>
+          <t>P05</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -667,10 +667,10 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>493.21</v>
+        <v>452.11</v>
       </c>
       <c r="E8" t="n">
-        <v>493.71</v>
+        <v>452.61</v>
       </c>
     </row>
     <row r="9">
@@ -679,7 +679,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>S11</t>
+          <t>S08</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -688,10 +688,10 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>509.31</v>
+        <v>453.01</v>
       </c>
       <c r="E9" t="n">
-        <v>510.81</v>
+        <v>454.51</v>
       </c>
     </row>
     <row r="10">
@@ -700,19 +700,670 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
+          <t>P04</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>拍照</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>454.61</v>
+      </c>
+      <c r="E10" t="n">
+        <v>455.11</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>P09</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>拍照</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>455.21</v>
+      </c>
+      <c r="E11" t="n">
+        <v>455.71</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>P03</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>拍照</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>456.01</v>
+      </c>
+      <c r="E12" t="n">
+        <v>456.51</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>P12</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>拍照</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>457.01</v>
+      </c>
+      <c r="E13" t="n">
+        <v>457.51</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>S07</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>射击</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>458.01</v>
+      </c>
+      <c r="E14" t="n">
+        <v>459.51</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>S09</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>射击</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>459.71</v>
+      </c>
+      <c r="E15" t="n">
+        <v>461.21</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>S03</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>射击</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>462.01</v>
+      </c>
+      <c r="E16" t="n">
+        <v>463.51</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>P11</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>拍照</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>463.81</v>
+      </c>
+      <c r="E17" t="n">
+        <v>464.31</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>S04</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>射击</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>464.41</v>
+      </c>
+      <c r="E18" t="n">
+        <v>465.91</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>P07</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>拍照</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>466.01</v>
+      </c>
+      <c r="E19" t="n">
+        <v>466.51</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>P16</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>拍照</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>466.61</v>
+      </c>
+      <c r="E20" t="n">
+        <v>467.11</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>P13</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>拍照</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>467.21</v>
+      </c>
+      <c r="E21" t="n">
+        <v>467.71</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>P06</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>拍照</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>467.81</v>
+      </c>
+      <c r="E22" t="n">
+        <v>468.31</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>P15</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>拍照</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>468.41</v>
+      </c>
+      <c r="E23" t="n">
+        <v>468.91</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>S02</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>射击</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>476.81</v>
+      </c>
+      <c r="E24" t="n">
+        <v>478.31</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>S01</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>射击</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
+        <v>478.51</v>
+      </c>
+      <c r="E25" t="n">
+        <v>480.01</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>P14</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>拍照</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
+        <v>480.51</v>
+      </c>
+      <c r="E26" t="n">
+        <v>481.01</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="n">
+        <v>26</v>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>P02</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>拍照</t>
+        </is>
+      </c>
+      <c r="D27" t="n">
+        <v>481.21</v>
+      </c>
+      <c r="E27" t="n">
+        <v>481.71</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="n">
+        <v>27</v>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>P06</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>拍照</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>481.81</v>
+      </c>
+      <c r="E28" t="n">
+        <v>482.31</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="n">
+        <v>28</v>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>P11</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>拍照</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
+        <v>492.41</v>
+      </c>
+      <c r="E29" t="n">
+        <v>492.91</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="n">
+        <v>29</v>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>P10</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>拍照</t>
+        </is>
+      </c>
+      <c r="D30" t="n">
+        <v>493.01</v>
+      </c>
+      <c r="E30" t="n">
+        <v>493.51</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="n">
+        <v>30</v>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>P03</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>拍照</t>
+        </is>
+      </c>
+      <c r="D31" t="n">
+        <v>493.61</v>
+      </c>
+      <c r="E31" t="n">
+        <v>494.11</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="n">
+        <v>31</v>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>P04</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>拍照</t>
+        </is>
+      </c>
+      <c r="D32" t="n">
+        <v>494.41</v>
+      </c>
+      <c r="E32" t="n">
+        <v>494.91</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="n">
+        <v>32</v>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>P01</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>拍照</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>508.41</v>
+      </c>
+      <c r="E33" t="n">
+        <v>508.91</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="n">
+        <v>33</v>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>P02</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>拍照</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
+        <v>509.01</v>
+      </c>
+      <c r="E34" t="n">
+        <v>509.51</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="n">
+        <v>34</v>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>S11</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>射击</t>
+        </is>
+      </c>
+      <c r="D35" t="n">
+        <v>515.8099999999999</v>
+      </c>
+      <c r="E35" t="n">
+        <v>517.3099999999999</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="n">
+        <v>35</v>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
           <t>S10</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
+      <c r="C36" t="inlineStr">
         <is>
           <t>射击</t>
         </is>
       </c>
-      <c r="D10" t="n">
+      <c r="D36" t="n">
         <v>525.51</v>
       </c>
-      <c r="E10" t="n">
+      <c r="E36" t="n">
         <v>527.01</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="n">
+        <v>36</v>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>P02</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>拍照</t>
+        </is>
+      </c>
+      <c r="D37" t="n">
+        <v>749.8099999999999</v>
+      </c>
+      <c r="E37" t="n">
+        <v>750.3099999999999</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="n">
+        <v>37</v>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>P05</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>拍照</t>
+        </is>
+      </c>
+      <c r="D38" t="n">
+        <v>750.41</v>
+      </c>
+      <c r="E38" t="n">
+        <v>750.91</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="n">
+        <v>38</v>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>S15</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>射击</t>
+        </is>
+      </c>
+      <c r="D39" t="n">
+        <v>751.01</v>
+      </c>
+      <c r="E39" t="n">
+        <v>752.51</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="n">
+        <v>39</v>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>S13</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>射击</t>
+        </is>
+      </c>
+      <c r="D40" t="n">
+        <v>762.01</v>
+      </c>
+      <c r="E40" t="n">
+        <v>763.51</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="n">
+        <v>40</v>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>S12</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>射击</t>
+        </is>
+      </c>
+      <c r="D41" t="n">
+        <v>807.8099999999999</v>
+      </c>
+      <c r="E41" t="n">
+        <v>809.3099999999999</v>
       </c>
     </row>
   </sheetData>

</xml_diff>